<commit_message>
Book1 H1 tags: more lookups
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4358,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -4992,30 +4992,30 @@
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>No page found for this part number by web search; not confident enough to name the appliance/part</t>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="4" t="inlineStr">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B186" s="4" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>W10314419</t>
         </is>
       </c>
-      <c r="C186" s="4" t="inlineStr"/>
-      <c r="D186" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E186" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C186" s="2" t="inlineStr"/>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5047,48 +5047,52 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="4" t="inlineStr">
+      <c r="A188" s="3" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B188" s="4" t="inlineStr">
+      <c r="B188" s="3" t="inlineStr">
         <is>
           <t>WPW10271740</t>
         </is>
       </c>
-      <c r="C188" s="4" t="inlineStr"/>
-      <c r="D188" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E188" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Control Board (No Overlay) - WPW10271740</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>ShopJimmy: range control board without overlay (WFE381LV series); sheet brand "LG" differs from part-number brand "Whirlpool"</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="4" t="inlineStr">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B189" s="4" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>WPW10271737</t>
         </is>
       </c>
-      <c r="C189" s="4" t="inlineStr"/>
-      <c r="D189" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E189" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C189" s="2" t="inlineStr"/>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5174,48 +5178,48 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="4" t="inlineStr">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B193" s="4" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>WP8507P226-60</t>
         </is>
       </c>
-      <c r="C193" s="4" t="inlineStr"/>
-      <c r="D193" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E193" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C193" s="2" t="inlineStr"/>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="4" t="inlineStr">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B194" s="4" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>DE92-02439F</t>
         </is>
       </c>
-      <c r="C194" s="4" t="inlineStr"/>
-      <c r="D194" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E194" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C194" s="2" t="inlineStr"/>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5274,25 +5278,25 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="4" t="inlineStr">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B197" s="4" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>MEE62306301</t>
         </is>
       </c>
-      <c r="C197" s="4" t="inlineStr"/>
-      <c r="D197" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E197" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C197" s="2" t="inlineStr"/>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5351,25 +5355,29 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="4" t="inlineStr">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B200" s="4" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>DG97-00053T</t>
         </is>
       </c>
-      <c r="C200" s="4" t="inlineStr"/>
-      <c r="D200" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E200" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Oven/Microwave Combo Drawer - DG97-00053T</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>samsungparts.com lists it as "Drawer" (oven/microwave combo); wording inconsistent; sheet brand "LG" differs from part-number brand "Samsung"</t>
         </is>
       </c>
     </row>
@@ -5455,232 +5463,248 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="4" t="inlineStr">
+      <c r="A204" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B204" s="4" t="inlineStr">
+      <c r="B204" s="2" t="inlineStr">
         <is>
           <t>AGM75309045</t>
         </is>
       </c>
-      <c r="C204" s="4" t="inlineStr"/>
-      <c r="D204" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E204" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>LG Range Parts Assembly - AGM75309045</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>lgparts.com: oven-range parts assembly; generic description</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="4" t="inlineStr">
+      <c r="A205" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B205" s="4" t="inlineStr">
+      <c r="B205" s="2" t="inlineStr">
         <is>
           <t>DG94-04148E</t>
         </is>
       </c>
-      <c r="C205" s="4" t="inlineStr"/>
-      <c r="D205" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E205" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C205" s="2" t="inlineStr"/>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="4" t="inlineStr">
+      <c r="A206" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B206" s="4" t="inlineStr">
+      <c r="B206" s="2" t="inlineStr">
         <is>
           <t>DE81-07021A</t>
         </is>
       </c>
-      <c r="C206" s="4" t="inlineStr"/>
-      <c r="D206" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E206" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Service Cooling Fan (110 CFM) - DE81-07021A</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>PartsWarehouse: Svc Fan Cooling 110 CFM; appliance not stated; sheet brand "Whirlpool" differs from part-number brand "Samsung"</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="4" t="inlineStr">
+      <c r="A207" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B207" s="4" t="inlineStr">
+      <c r="B207" s="2" t="inlineStr">
         <is>
           <t>DE81-04526A</t>
         </is>
       </c>
-      <c r="C207" s="4" t="inlineStr"/>
-      <c r="D207" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E207" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C207" s="2" t="inlineStr"/>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="4" t="inlineStr">
+      <c r="A208" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B208" s="4" t="inlineStr">
+      <c r="B208" s="3" t="inlineStr">
         <is>
           <t>AGM30025503</t>
         </is>
       </c>
-      <c r="C208" s="4" t="inlineStr"/>
-      <c r="D208" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E208" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Control Panel - AGM30025503</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>lgparts.com: range control panel; sheet brand "Whirlpool" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="4" t="inlineStr">
+      <c r="A209" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B209" s="4" t="inlineStr">
+      <c r="B209" s="3" t="inlineStr">
         <is>
           <t>EBR87050406</t>
         </is>
       </c>
-      <c r="C209" s="4" t="inlineStr"/>
-      <c r="D209" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E209" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Main Power Control Board - EBR87050406</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts/genuinereplacementparts: range PCB assembly (LRE4211ST etc.); sheet brand "Whirlpool" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="4" t="inlineStr">
+      <c r="A210" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B210" s="4" t="inlineStr">
+      <c r="B210" s="2" t="inlineStr">
         <is>
           <t>W11295990</t>
         </is>
       </c>
-      <c r="C210" s="4" t="inlineStr"/>
-      <c r="D210" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E210" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C210" s="2" t="inlineStr"/>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="4" t="inlineStr">
+      <c r="A211" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B211" s="4" t="inlineStr">
+      <c r="B211" s="2" t="inlineStr">
         <is>
           <t>EBR87050404</t>
         </is>
       </c>
-      <c r="C211" s="4" t="inlineStr"/>
-      <c r="D211" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E211" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C211" s="2" t="inlineStr"/>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="4" t="inlineStr">
+      <c r="A212" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B212" s="4" t="inlineStr">
+      <c r="B212" s="2" t="inlineStr">
         <is>
           <t>EBR87050401</t>
         </is>
       </c>
-      <c r="C212" s="4" t="inlineStr"/>
-      <c r="D212" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E212" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C212" s="2" t="inlineStr"/>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="4" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B213" s="4" t="inlineStr">
+      <c r="B213" s="2" t="inlineStr">
         <is>
           <t>EBR85707901</t>
         </is>
       </c>
-      <c r="C213" s="4" t="inlineStr"/>
-      <c r="D213" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E213" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C213" s="2" t="inlineStr"/>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5712,25 +5736,25 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="4" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B215" s="4" t="inlineStr">
+      <c r="B215" s="2" t="inlineStr">
         <is>
           <t>DG94-01301E</t>
         </is>
       </c>
-      <c r="C215" s="4" t="inlineStr"/>
-      <c r="D215" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E215" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C215" s="2" t="inlineStr"/>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5762,25 +5786,29 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="4" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B217" s="4" t="inlineStr">
+      <c r="B217" s="2" t="inlineStr">
         <is>
           <t>ACM75039302</t>
         </is>
       </c>
-      <c r="C217" s="4" t="inlineStr"/>
-      <c r="D217" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E217" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>LG Sub Controller Assembly - ACM75039302</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>lgparts.com: sub controller assembly; appliance not clearly stated; sheet brand "Bertazzoni" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
@@ -5812,48 +5840,52 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="4" t="inlineStr">
+      <c r="A219" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B219" s="4" t="inlineStr">
+      <c r="B219" s="3" t="inlineStr">
         <is>
           <t>W11122543</t>
         </is>
       </c>
-      <c r="C219" s="4" t="inlineStr"/>
-      <c r="D219" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E219" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Electric Control - W11122543</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply: electric control for range (listed as W11122543C); sheet brand "Bertazzoni" differs from part-number brand "Whirlpool"</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="4" t="inlineStr">
+      <c r="A220" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B220" s="4" t="inlineStr">
+      <c r="B220" s="2" t="inlineStr">
         <is>
           <t>W11122531</t>
         </is>
       </c>
-      <c r="C220" s="4" t="inlineStr"/>
-      <c r="D220" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E220" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C220" s="2" t="inlineStr"/>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -5885,163 +5917,167 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="4" t="inlineStr">
+      <c r="A222" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B222" s="4" t="inlineStr">
+      <c r="B222" s="2" t="inlineStr">
         <is>
           <t>DG94-01301G</t>
         </is>
       </c>
-      <c r="C222" s="4" t="inlineStr"/>
-      <c r="D222" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E222" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C222" s="2" t="inlineStr"/>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="4" t="inlineStr">
+      <c r="A223" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B223" s="4" t="inlineStr">
+      <c r="B223" s="2" t="inlineStr">
         <is>
           <t>DG92-01198F</t>
         </is>
       </c>
-      <c r="C223" s="4" t="inlineStr"/>
-      <c r="D223" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E223" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C223" s="2" t="inlineStr"/>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="4" t="inlineStr">
+      <c r="A224" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B224" s="4" t="inlineStr">
+      <c r="B224" s="2" t="inlineStr">
         <is>
           <t>DG94-01548B</t>
         </is>
       </c>
-      <c r="C224" s="4" t="inlineStr"/>
-      <c r="D224" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E224" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C224" s="2" t="inlineStr"/>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="4" t="inlineStr">
+      <c r="A225" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B225" s="4" t="inlineStr">
+      <c r="B225" s="2" t="inlineStr">
         <is>
           <t>DG94-01545B</t>
         </is>
       </c>
-      <c r="C225" s="4" t="inlineStr"/>
-      <c r="D225" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E225" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C225" s="2" t="inlineStr"/>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="4" t="inlineStr">
+      <c r="A226" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B226" s="4" t="inlineStr">
+      <c r="B226" s="2" t="inlineStr">
         <is>
           <t>DG94-03952S</t>
         </is>
       </c>
-      <c r="C226" s="4" t="inlineStr"/>
-      <c r="D226" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Control Box Module Assembly - DG94-03952S</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>samsungparts.com: assy control box-module; appliance not stated; sheet brand "Bertazzoni" differs from part-number brand "Samsung"</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="4" t="inlineStr">
+      <c r="A227" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B227" s="4" t="inlineStr">
+      <c r="B227" s="2" t="inlineStr">
         <is>
           <t>DG94-04664P</t>
         </is>
       </c>
-      <c r="C227" s="4" t="inlineStr"/>
-      <c r="D227" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E227" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C227" s="2" t="inlineStr"/>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="4" t="inlineStr">
+      <c r="A228" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B228" s="4" t="inlineStr">
+      <c r="B228" s="2" t="inlineStr">
         <is>
           <t>Z350251</t>
         </is>
       </c>
-      <c r="C228" s="4" t="inlineStr"/>
-      <c r="D228" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E228" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C228" s="2" t="inlineStr"/>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -6193,140 +6229,140 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="4" t="inlineStr">
+      <c r="A236" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B236" s="4" t="inlineStr">
+      <c r="B236" s="2" t="inlineStr">
         <is>
           <t>128006-DA</t>
         </is>
       </c>
-      <c r="C236" s="4" t="inlineStr"/>
-      <c r="D236" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C236" s="2" t="inlineStr"/>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="4" t="inlineStr">
+      <c r="A237" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B237" s="4" t="inlineStr">
+      <c r="B237" s="2" t="inlineStr">
         <is>
           <t>1080923-DA</t>
         </is>
       </c>
-      <c r="C237" s="4" t="inlineStr"/>
-      <c r="D237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E237" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C237" s="2" t="inlineStr"/>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="4" t="inlineStr">
+      <c r="A238" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B238" s="4" t="inlineStr">
+      <c r="B238" s="2" t="inlineStr">
         <is>
           <t>1080921-DA</t>
         </is>
       </c>
-      <c r="C238" s="4" t="inlineStr"/>
-      <c r="D238" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E238" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C238" s="2" t="inlineStr"/>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="4" t="inlineStr">
+      <c r="A239" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B239" s="4" t="inlineStr">
+      <c r="B239" s="2" t="inlineStr">
         <is>
           <t>128017-DA</t>
         </is>
       </c>
-      <c r="C239" s="4" t="inlineStr"/>
-      <c r="D239" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E239" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C239" s="2" t="inlineStr"/>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="4" t="inlineStr">
+      <c r="A240" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B240" s="4" t="inlineStr">
+      <c r="B240" s="2" t="inlineStr">
         <is>
           <t>128023-DA</t>
         </is>
       </c>
-      <c r="C240" s="4" t="inlineStr"/>
-      <c r="D240" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E240" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C240" s="2" t="inlineStr"/>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="4" t="inlineStr">
+      <c r="A241" s="2" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B241" s="4" t="inlineStr">
+      <c r="B241" s="2" t="inlineStr">
         <is>
           <t>128032-DA</t>
         </is>
       </c>
-      <c r="C241" s="4" t="inlineStr"/>
-      <c r="D241" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E241" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C241" s="2" t="inlineStr"/>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -6415,25 +6451,25 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="4" t="inlineStr">
+      <c r="A246" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B246" s="4" t="inlineStr">
+      <c r="B246" s="2" t="inlineStr">
         <is>
           <t>Z180301</t>
         </is>
       </c>
-      <c r="C246" s="4" t="inlineStr"/>
-      <c r="D246" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E246" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C246" s="2" t="inlineStr"/>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -6879,25 +6915,29 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="4" t="inlineStr">
+      <c r="A268" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B268" s="4" t="inlineStr">
+      <c r="B268" s="3" t="inlineStr">
         <is>
           <t>WB27K10423</t>
         </is>
       </c>
-      <c r="C268" s="4" t="inlineStr"/>
-      <c r="D268" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E268" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board - WB27K10423</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply: control board for range; sheet brand "Frigidaire" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -6992,48 +7032,56 @@
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="4" t="inlineStr">
+      <c r="A273" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B273" s="4" t="inlineStr">
+      <c r="B273" s="3" t="inlineStr">
         <is>
           <t>WB27X25329</t>
         </is>
       </c>
-      <c r="C273" s="4" t="inlineStr"/>
-      <c r="D273" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E273" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board (No Overlay) - WB27X25329</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>ShopJimmy: range control board without overlay; sheet brand "Bosch" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="4" t="inlineStr">
+      <c r="A274" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B274" s="4" t="inlineStr">
+      <c r="B274" s="3" t="inlineStr">
         <is>
           <t>WB27X25332</t>
         </is>
       </c>
-      <c r="C274" s="4" t="inlineStr"/>
-      <c r="D274" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E274" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board - WB27X25332</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts: control board, fits PGS920SEF1SS range; sheet brand "Bosch" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -7422,25 +7470,29 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="4" t="inlineStr">
+      <c r="A293" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B293" s="4" t="inlineStr">
+      <c r="B293" s="2" t="inlineStr">
         <is>
           <t>WB27X32205</t>
         </is>
       </c>
-      <c r="C293" s="4" t="inlineStr"/>
-      <c r="D293" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E293" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>GE Range Control Panel - WB27X32205</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>eBay listing: double gas oven control panel (single source); sheet brand "Frigidaire" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -7619,25 +7671,29 @@
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="4" t="inlineStr">
+      <c r="A302" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B302" s="4" t="inlineStr">
+      <c r="B302" s="3" t="inlineStr">
         <is>
           <t>WB20X126</t>
         </is>
       </c>
-      <c r="C302" s="4" t="inlineStr"/>
-      <c r="D302" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E302" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Valve - WB20X126</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E302" s="3" t="inlineStr">
+        <is>
+          <t>GE Appliances / HD Supply: gas range control valve; sheet brand "Frigidaire" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -7774,25 +7830,29 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="4" t="inlineStr">
+      <c r="A309" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B309" s="4" t="inlineStr">
+      <c r="B309" s="3" t="inlineStr">
         <is>
           <t>WB23T10024</t>
         </is>
       </c>
-      <c r="C309" s="4" t="inlineStr"/>
-      <c r="D309" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E309" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board - WB23T10024</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>geapplianceparts.com: Range Control Board; sheet brand "Frigidaire" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -7824,48 +7884,52 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="4" t="inlineStr">
+      <c r="A311" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B311" s="4" t="inlineStr">
+      <c r="B311" s="3" t="inlineStr">
         <is>
           <t>WB19K10061</t>
         </is>
       </c>
-      <c r="C311" s="4" t="inlineStr"/>
-      <c r="D311" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E311" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Oven Relay Control Board - WB19K10061</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts: GE range oven relay control board; sheet brand "Frigidaire" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="4" t="inlineStr">
+      <c r="A312" s="2" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B312" s="4" t="inlineStr">
+      <c r="B312" s="2" t="inlineStr">
         <is>
           <t>WB57K10128</t>
         </is>
       </c>
-      <c r="C312" s="4" t="inlineStr"/>
-      <c r="D312" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E312" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C312" s="2" t="inlineStr"/>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -8380,117 +8444,133 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="4" t="inlineStr">
+      <c r="A337" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B337" s="4" t="inlineStr">
+      <c r="B337" s="2" t="inlineStr">
         <is>
           <t>WB48X23580</t>
         </is>
       </c>
-      <c r="C337" s="4" t="inlineStr"/>
-      <c r="D337" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E337" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C337" s="2" t="inlineStr"/>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="338">
-      <c r="A338" s="4" t="inlineStr">
+      <c r="A338" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B338" s="4" t="inlineStr">
+      <c r="B338" s="3" t="inlineStr">
         <is>
           <t>WB56X33178</t>
         </is>
       </c>
-      <c r="C338" s="4" t="inlineStr"/>
-      <c r="D338" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E338" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C338" s="3" t="inlineStr">
+        <is>
+          <t>GE Wall Oven Stainless Steel Outer Door Assembly - WB56X33178</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="inlineStr">
+        <is>
+          <t>iFixit: outer door assembly, fits JT5000/PT9050 series; sheet brand "Bosch" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="4" t="inlineStr">
+      <c r="A339" s="2" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B339" s="4" t="inlineStr">
+      <c r="B339" s="2" t="inlineStr">
         <is>
           <t>WB27X35131</t>
         </is>
       </c>
-      <c r="C339" s="4" t="inlineStr"/>
-      <c r="D339" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E339" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>GE Module Board - WB27X35131</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>GE Appliance Parts: module board; appliance not stated; sheet brand "Blomberg" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="340">
-      <c r="A340" s="4" t="inlineStr">
+      <c r="A340" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B340" s="4" t="inlineStr">
+      <c r="B340" s="2" t="inlineStr">
         <is>
           <t>WB56X38529</t>
         </is>
       </c>
-      <c r="C340" s="4" t="inlineStr"/>
-      <c r="D340" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E340" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>GE Door Parts Assembly - WB56X38529</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>GE Appliance Parts: Parts Assembly-Door; appliance not stated; sheet brand "LG" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="341">
-      <c r="A341" s="4" t="inlineStr">
+      <c r="A341" s="2" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B341" s="4" t="inlineStr">
+      <c r="B341" s="2" t="inlineStr">
         <is>
           <t>WB56X38545</t>
         </is>
       </c>
-      <c r="C341" s="4" t="inlineStr"/>
-      <c r="D341" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E341" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>GE Door Assembly - WB56X38545</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>GE Appliance Parts: Door Assembly; appliance not stated; sheet brand "LG" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -8522,25 +8602,29 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="4" t="inlineStr">
+      <c r="A343" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B343" s="4" t="inlineStr">
+      <c r="B343" s="2" t="inlineStr">
         <is>
           <t>WB27X37850</t>
         </is>
       </c>
-      <c r="C343" s="4" t="inlineStr"/>
-      <c r="D343" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E343" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>GE Oven Control (RSC15) - WB27X37850</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>eBay listing: GEH oven control RSC15 (single source); sheet brand "Bosch" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -8881,25 +8965,29 @@
       </c>
     </row>
     <row r="360">
-      <c r="A360" s="4" t="inlineStr">
+      <c r="A360" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B360" s="4" t="inlineStr">
+      <c r="B360" s="3" t="inlineStr">
         <is>
           <t>AGM30025501</t>
         </is>
       </c>
-      <c r="C360" s="4" t="inlineStr"/>
-      <c r="D360" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E360" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C360" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Control Panel Assembly - AGM30025501</t>
+        </is>
+      </c>
+      <c r="D360" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E360" s="3" t="inlineStr">
+        <is>
+          <t>lgparts.com / HNK Parts: range control panel assembly; sheet brand "Bosch" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
@@ -8931,25 +9019,25 @@
       </c>
     </row>
     <row r="362">
-      <c r="A362" s="4" t="inlineStr">
+      <c r="A362" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B362" s="4" t="inlineStr">
+      <c r="B362" s="2" t="inlineStr">
         <is>
           <t>WP6610457</t>
         </is>
       </c>
-      <c r="C362" s="4" t="inlineStr"/>
-      <c r="D362" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E362" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C362" s="2" t="inlineStr"/>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -9907,25 +9995,25 @@
       </c>
     </row>
     <row r="408">
-      <c r="A408" s="4" t="inlineStr">
+      <c r="A408" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B408" s="4" t="inlineStr">
+      <c r="B408" s="2" t="inlineStr">
         <is>
           <t>128026-DA</t>
         </is>
       </c>
-      <c r="C408" s="4" t="inlineStr"/>
-      <c r="D408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C408" s="2" t="inlineStr"/>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -9978,48 +10066,48 @@
       </c>
     </row>
     <row r="411">
-      <c r="A411" s="4" t="inlineStr">
+      <c r="A411" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B411" s="4" t="inlineStr">
+      <c r="B411" s="2" t="inlineStr">
         <is>
           <t>1080943-DA</t>
         </is>
       </c>
-      <c r="C411" s="4" t="inlineStr"/>
-      <c r="D411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C411" s="2" t="inlineStr"/>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E411" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="412">
-      <c r="A412" s="4" t="inlineStr">
+      <c r="A412" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B412" s="4" t="inlineStr">
+      <c r="B412" s="2" t="inlineStr">
         <is>
           <t>128024-DA</t>
         </is>
       </c>
-      <c r="C412" s="4" t="inlineStr"/>
-      <c r="D412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C412" s="2" t="inlineStr"/>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10045,25 +10133,25 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" s="4" t="inlineStr">
+      <c r="A414" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B414" s="4" t="inlineStr">
+      <c r="B414" s="2" t="inlineStr">
         <is>
           <t>Z160143</t>
         </is>
       </c>
-      <c r="C414" s="4" t="inlineStr"/>
-      <c r="D414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C414" s="2" t="inlineStr"/>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -11512,78 +11600,90 @@
       </c>
     </row>
     <row r="485">
-      <c r="A485" s="4" t="n"/>
-      <c r="B485" s="4" t="inlineStr">
+      <c r="A485" s="2" t="n"/>
+      <c r="B485" s="2" t="inlineStr">
         <is>
           <t>WB27X42946</t>
         </is>
       </c>
-      <c r="C485" s="4" t="inlineStr"/>
-      <c r="D485" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E485" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>GE Glass &amp; Touch Board Assembly - WB27X42946</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>iFixit listing; appliance not stated</t>
         </is>
       </c>
     </row>
     <row r="486">
-      <c r="A486" s="4" t="n"/>
-      <c r="B486" s="4" t="inlineStr">
+      <c r="A486" s="3" t="n"/>
+      <c r="B486" s="3" t="inlineStr">
         <is>
           <t>WB27X31709</t>
         </is>
       </c>
-      <c r="C486" s="4" t="inlineStr"/>
-      <c r="D486" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E486" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Glass &amp; Touch Board Assembly - WB27X31709</t>
+        </is>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>GE Appliance Parts / ShopJimmy: range glass touchpad assembly</t>
         </is>
       </c>
     </row>
     <row r="487">
-      <c r="A487" s="4" t="n"/>
-      <c r="B487" s="4" t="inlineStr">
+      <c r="A487" s="3" t="n"/>
+      <c r="B487" s="3" t="inlineStr">
         <is>
           <t>WB27X25332</t>
         </is>
       </c>
-      <c r="C487" s="4" t="inlineStr"/>
-      <c r="D487" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E487" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C487" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board - WB27X25332</t>
+        </is>
+      </c>
+      <c r="D487" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E487" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts: control board, fits PGS920SEF1SS range</t>
         </is>
       </c>
     </row>
     <row r="488">
-      <c r="A488" s="4" t="n"/>
-      <c r="B488" s="4" t="inlineStr">
+      <c r="A488" s="2" t="n"/>
+      <c r="B488" s="2" t="inlineStr">
         <is>
           <t>WB56X25765</t>
         </is>
       </c>
-      <c r="C488" s="4" t="inlineStr"/>
-      <c r="D488" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E488" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C488" s="2" t="inlineStr"/>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -11656,154 +11756,174 @@
       </c>
     </row>
     <row r="493">
-      <c r="A493" s="4" t="n"/>
-      <c r="B493" s="4" t="inlineStr">
+      <c r="A493" s="2" t="n"/>
+      <c r="B493" s="2" t="inlineStr">
         <is>
           <t>WB27X43578</t>
         </is>
       </c>
-      <c r="C493" s="4" t="inlineStr"/>
-      <c r="D493" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E493" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C493" s="2" t="inlineStr"/>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="494">
-      <c r="A494" s="4" t="n"/>
-      <c r="B494" s="4" t="inlineStr">
+      <c r="A494" s="3" t="n"/>
+      <c r="B494" s="3" t="inlineStr">
         <is>
           <t>WB27K10423</t>
         </is>
       </c>
-      <c r="C494" s="4" t="inlineStr"/>
-      <c r="D494" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E494" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C494" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Board - WB27K10423</t>
+        </is>
+      </c>
+      <c r="D494" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E494" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply: control board for range</t>
         </is>
       </c>
     </row>
     <row r="495">
-      <c r="A495" s="4" t="n"/>
-      <c r="B495" s="4" t="inlineStr">
+      <c r="A495" s="2" t="n"/>
+      <c r="B495" s="2" t="inlineStr">
         <is>
           <t>MGC64258906</t>
         </is>
       </c>
-      <c r="C495" s="4" t="inlineStr"/>
-      <c r="D495" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E495" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C495" s="2" t="inlineStr"/>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="496">
-      <c r="A496" s="4" t="n"/>
-      <c r="B496" s="4" t="inlineStr">
+      <c r="A496" s="2" t="n"/>
+      <c r="B496" s="2" t="inlineStr">
         <is>
           <t>MEB63654003</t>
         </is>
       </c>
-      <c r="C496" s="4" t="inlineStr"/>
-      <c r="D496" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E496" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C496" s="2" t="inlineStr"/>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="497">
-      <c r="A497" s="4" t="n"/>
-      <c r="B497" s="4" t="inlineStr">
+      <c r="A497" s="3" t="n"/>
+      <c r="B497" s="3" t="inlineStr">
         <is>
           <t>AHT74673902</t>
         </is>
       </c>
-      <c r="C497" s="4" t="inlineStr"/>
-      <c r="D497" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E497" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C497" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Shelf Assembly - AHT74673902</t>
+        </is>
+      </c>
+      <c r="D497" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E497" s="3" t="inlineStr">
+        <is>
+          <t>lgparts.com: oven-range shelf assembly</t>
         </is>
       </c>
     </row>
     <row r="498">
-      <c r="A498" s="4" t="n"/>
-      <c r="B498" s="4" t="inlineStr">
+      <c r="A498" s="2" t="n"/>
+      <c r="B498" s="2" t="inlineStr">
         <is>
           <t>AJX74385101</t>
         </is>
       </c>
-      <c r="C498" s="4" t="inlineStr"/>
-      <c r="D498" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E498" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>LG Window Assembly - AJX74385101</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>lgparts.com: window assembly; appliance not stated</t>
         </is>
       </c>
     </row>
     <row r="499">
-      <c r="A499" s="4" t="n"/>
-      <c r="B499" s="4" t="inlineStr">
+      <c r="A499" s="2" t="n"/>
+      <c r="B499" s="2" t="inlineStr">
         <is>
           <t>AED74352702</t>
         </is>
       </c>
-      <c r="C499" s="4" t="inlineStr"/>
-      <c r="D499" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E499" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>LG Handle Assembly - AED74352702</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>lgparts.com: handle assembly; appliance not stated</t>
         </is>
       </c>
     </row>
     <row r="500">
-      <c r="A500" s="4" t="n"/>
-      <c r="B500" s="4" t="inlineStr">
+      <c r="A500" s="2" t="n"/>
+      <c r="B500" s="2" t="inlineStr">
         <is>
           <t>MKC66399505</t>
         </is>
       </c>
-      <c r="C500" s="4" t="inlineStr"/>
-      <c r="D500" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E500" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>LG Glass Window - MKC66399505</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>lgparts.com: glass window (sibling parts are oven-range windows)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1: complete title pass over all 499 rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,11 +46,6 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7307,25 +7301,25 @@
       </c>
     </row>
     <row r="280">
-      <c r="A280" s="4" t="inlineStr">
+      <c r="A280" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B280" s="4" t="inlineStr">
+      <c r="B280" s="2" t="inlineStr">
         <is>
           <t>618624</t>
         </is>
       </c>
-      <c r="C280" s="4" t="inlineStr"/>
-      <c r="D280" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E280" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C280" s="2" t="inlineStr"/>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -9140,25 +9134,25 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" s="4" t="inlineStr">
+      <c r="A355" s="2" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B355" s="4" t="inlineStr">
+      <c r="B355" s="2" t="inlineStr">
         <is>
           <t>669416</t>
         </is>
       </c>
-      <c r="C355" s="4" t="inlineStr"/>
-      <c r="D355" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E355" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C355" s="2" t="inlineStr"/>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -9942,25 +9936,25 @@
       </c>
     </row>
     <row r="389">
-      <c r="A389" s="4" t="inlineStr">
+      <c r="A389" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B389" s="4" t="inlineStr">
+      <c r="B389" s="2" t="inlineStr">
         <is>
           <t>260605044</t>
         </is>
       </c>
-      <c r="C389" s="4" t="inlineStr"/>
-      <c r="D389" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E389" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C389" s="2" t="inlineStr"/>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10034,25 +10028,25 @@
       </c>
     </row>
     <row r="393">
-      <c r="A393" s="4" t="inlineStr">
+      <c r="A393" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B393" s="4" t="inlineStr">
+      <c r="B393" s="2" t="inlineStr">
         <is>
           <t>267600080</t>
         </is>
       </c>
-      <c r="C393" s="4" t="inlineStr"/>
-      <c r="D393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C393" s="2" t="inlineStr"/>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10172,25 +10166,25 @@
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="4" t="inlineStr">
+      <c r="A399" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B399" s="4" t="inlineStr">
+      <c r="B399" s="2" t="inlineStr">
         <is>
           <t>128003</t>
         </is>
       </c>
-      <c r="C399" s="4" t="inlineStr"/>
-      <c r="D399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C399" s="2" t="inlineStr"/>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10364,25 +10358,25 @@
       </c>
     </row>
     <row r="407">
-      <c r="A407" s="4" t="inlineStr">
+      <c r="A407" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B407" s="4" t="inlineStr">
+      <c r="B407" s="2" t="inlineStr">
         <is>
           <t>128036-DA</t>
         </is>
       </c>
-      <c r="C407" s="4" t="inlineStr"/>
-      <c r="D407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C407" s="2" t="inlineStr"/>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10698,71 +10692,71 @@
       </c>
     </row>
     <row r="421">
-      <c r="A421" s="4" t="inlineStr">
+      <c r="A421" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B421" s="4" t="inlineStr">
+      <c r="B421" s="2" t="inlineStr">
         <is>
           <t>125134</t>
         </is>
       </c>
-      <c r="C421" s="4" t="inlineStr"/>
-      <c r="D421" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E421" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C421" s="2" t="inlineStr"/>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="422">
-      <c r="A422" s="4" t="inlineStr">
+      <c r="A422" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B422" s="4" t="inlineStr">
+      <c r="B422" s="2" t="inlineStr">
         <is>
           <t>125345</t>
         </is>
       </c>
-      <c r="C422" s="4" t="inlineStr"/>
-      <c r="D422" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E422" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C422" s="2" t="inlineStr"/>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="423">
-      <c r="A423" s="4" t="inlineStr">
+      <c r="A423" s="2" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B423" s="4" t="inlineStr">
+      <c r="B423" s="2" t="inlineStr">
         <is>
           <t>125322</t>
         </is>
       </c>
-      <c r="C423" s="4" t="inlineStr"/>
-      <c r="D423" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E423" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C423" s="2" t="inlineStr"/>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10794,25 +10788,25 @@
       </c>
     </row>
     <row r="425">
-      <c r="A425" s="4" t="inlineStr">
+      <c r="A425" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B425" s="4" t="inlineStr">
+      <c r="B425" s="2" t="inlineStr">
         <is>
           <t>125170</t>
         </is>
       </c>
-      <c r="C425" s="4" t="inlineStr"/>
-      <c r="D425" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E425" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C425" s="2" t="inlineStr"/>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -10844,163 +10838,163 @@
       </c>
     </row>
     <row r="427">
-      <c r="A427" s="4" t="inlineStr">
+      <c r="A427" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B427" s="4" t="inlineStr">
+      <c r="B427" s="2" t="inlineStr">
         <is>
           <t>125309</t>
         </is>
       </c>
-      <c r="C427" s="4" t="inlineStr"/>
-      <c r="D427" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E427" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C427" s="2" t="inlineStr"/>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="428">
-      <c r="A428" s="4" t="inlineStr">
+      <c r="A428" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B428" s="4" t="inlineStr">
+      <c r="B428" s="2" t="inlineStr">
         <is>
           <t>125321</t>
         </is>
       </c>
-      <c r="C428" s="4" t="inlineStr"/>
-      <c r="D428" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E428" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C428" s="2" t="inlineStr"/>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="429">
-      <c r="A429" s="4" t="inlineStr">
+      <c r="A429" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B429" s="4" t="inlineStr">
+      <c r="B429" s="2" t="inlineStr">
         <is>
           <t>125341</t>
         </is>
       </c>
-      <c r="C429" s="4" t="inlineStr"/>
-      <c r="D429" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E429" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C429" s="2" t="inlineStr"/>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="430">
-      <c r="A430" s="4" t="inlineStr">
+      <c r="A430" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B430" s="4" t="inlineStr">
+      <c r="B430" s="2" t="inlineStr">
         <is>
           <t>125346</t>
         </is>
       </c>
-      <c r="C430" s="4" t="inlineStr"/>
-      <c r="D430" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E430" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C430" s="2" t="inlineStr"/>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="431">
-      <c r="A431" s="4" t="inlineStr">
+      <c r="A431" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B431" s="4" t="inlineStr">
+      <c r="B431" s="2" t="inlineStr">
         <is>
           <t>200536</t>
         </is>
       </c>
-      <c r="C431" s="4" t="inlineStr"/>
-      <c r="D431" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E431" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C431" s="2" t="inlineStr"/>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="432">
-      <c r="A432" s="4" t="inlineStr">
+      <c r="A432" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B432" s="4" t="inlineStr">
+      <c r="B432" s="2" t="inlineStr">
         <is>
           <t>125162</t>
         </is>
       </c>
-      <c r="C432" s="4" t="inlineStr"/>
-      <c r="D432" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E432" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C432" s="2" t="inlineStr"/>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="433">
-      <c r="A433" s="4" t="inlineStr">
+      <c r="A433" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B433" s="4" t="inlineStr">
+      <c r="B433" s="2" t="inlineStr">
         <is>
           <t>125187</t>
         </is>
       </c>
-      <c r="C433" s="4" t="inlineStr"/>
-      <c r="D433" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E433" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C433" s="2" t="inlineStr"/>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -11032,117 +11026,117 @@
       </c>
     </row>
     <row r="435">
-      <c r="A435" s="4" t="inlineStr">
+      <c r="A435" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B435" s="4" t="inlineStr">
+      <c r="B435" s="2" t="inlineStr">
         <is>
           <t>125317</t>
         </is>
       </c>
-      <c r="C435" s="4" t="inlineStr"/>
-      <c r="D435" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E435" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C435" s="2" t="inlineStr"/>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="436">
-      <c r="A436" s="4" t="inlineStr">
+      <c r="A436" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B436" s="4" t="inlineStr">
+      <c r="B436" s="2" t="inlineStr">
         <is>
           <t>125323</t>
         </is>
       </c>
-      <c r="C436" s="4" t="inlineStr"/>
-      <c r="D436" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E436" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C436" s="2" t="inlineStr"/>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="437">
-      <c r="A437" s="4" t="inlineStr">
+      <c r="A437" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B437" s="4" t="inlineStr">
+      <c r="B437" s="2" t="inlineStr">
         <is>
           <t>125307</t>
         </is>
       </c>
-      <c r="C437" s="4" t="inlineStr"/>
-      <c r="D437" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E437" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C437" s="2" t="inlineStr"/>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="438">
-      <c r="A438" s="4" t="inlineStr">
+      <c r="A438" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B438" s="4" t="inlineStr">
+      <c r="B438" s="2" t="inlineStr">
         <is>
           <t>125318</t>
         </is>
       </c>
-      <c r="C438" s="4" t="inlineStr"/>
-      <c r="D438" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E438" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C438" s="2" t="inlineStr"/>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="439">
-      <c r="A439" s="4" t="inlineStr">
+      <c r="A439" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B439" s="4" t="inlineStr">
+      <c r="B439" s="2" t="inlineStr">
         <is>
           <t>410701</t>
         </is>
       </c>
-      <c r="C439" s="4" t="inlineStr"/>
-      <c r="D439" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E439" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C439" s="2" t="inlineStr"/>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
@@ -11174,71 +11168,75 @@
       </c>
     </row>
     <row r="441">
-      <c r="A441" s="4" t="inlineStr">
+      <c r="A441" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B441" s="4" t="inlineStr">
+      <c r="B441" s="2" t="inlineStr">
         <is>
           <t>125339</t>
         </is>
       </c>
-      <c r="C441" s="4" t="inlineStr"/>
-      <c r="D441" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E441" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C441" s="2" t="inlineStr"/>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>
     <row r="442">
-      <c r="A442" s="4" t="inlineStr">
+      <c r="A442" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B442" s="4" t="inlineStr">
+      <c r="B442" s="2" t="inlineStr">
         <is>
           <t>1080448</t>
         </is>
       </c>
-      <c r="C442" s="4" t="inlineStr"/>
-      <c r="D442" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E442" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>Bertazzoni Oven Door (Beige) - 1080448</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>Parts Town listing; fitment not stated; sheet brand "Electrolux" differs from part-number brand "Bertazzoni"</t>
         </is>
       </c>
     </row>
     <row r="443">
-      <c r="A443" s="4" t="inlineStr">
+      <c r="A443" s="2" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B443" s="4" t="inlineStr">
+      <c r="B443" s="2" t="inlineStr">
         <is>
           <t>1080442</t>
         </is>
       </c>
-      <c r="C443" s="4" t="inlineStr"/>
-      <c r="D443" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E443" s="4" t="inlineStr">
-        <is>
-          <t>Not searched yet</t>
+      <c r="C443" s="2" t="inlineStr"/>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1: second search pass adds 5 titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -540,25 +540,29 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>W10245805</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Main Top Assembly - W10245805</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply exact-number listing: main top assembly for range; also fits some Maytag/Amana/IKEA models (2nd pass)</t>
         </is>
       </c>
     </row>
@@ -700,15 +704,19 @@
           <t>W11122551</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Range Electronic Control - W11122551</t>
+        </is>
+      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+          <t>HD Supply lists "Electric Control For Range, Part# W11122551c" (vendor adds c suffix; replaces W10887916); fitment not stated (2nd pass); sheet brand "LG" differs from part-number brand "Whirlpool"</t>
         </is>
       </c>
     </row>
@@ -7182,25 +7190,29 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="inlineStr">
+      <c r="A275" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B275" s="2" t="inlineStr">
+      <c r="B275" s="3" t="inlineStr">
         <is>
           <t>5304503758</t>
         </is>
       </c>
-      <c r="C275" s="2" t="inlineStr"/>
-      <c r="D275" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E275" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Electronic Oven Control Board - 5304503758</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing: genuine Frigidaire electronic oven controller; fitment not stated (2nd pass); sheet brand "Bosch" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -8162,25 +8174,29 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="inlineStr">
+      <c r="A315" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B315" s="2" t="inlineStr">
+      <c r="B315" s="3" t="inlineStr">
         <is>
           <t>316462864</t>
         </is>
       </c>
-      <c r="C315" s="2" t="inlineStr"/>
-      <c r="D315" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E315" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Oven Control Board (Controller) - 316462864</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>Fix.com listing "CONTROLLER 316462864", Frigidaire ranges; supersedes AP4454715/316462891 (2nd pass)</t>
         </is>
       </c>
     </row>
@@ -12165,21 +12181,25 @@
       </c>
     </row>
     <row r="484">
-      <c r="A484" s="2" t="n"/>
-      <c r="B484" s="2" t="inlineStr">
+      <c r="A484" s="3" t="n"/>
+      <c r="B484" s="3" t="inlineStr">
         <is>
           <t>5304503758</t>
         </is>
       </c>
-      <c r="C484" s="2" t="inlineStr"/>
-      <c r="D484" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E484" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C484" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Electronic Oven Control Board - 5304503758</t>
+        </is>
+      </c>
+      <c r="D484" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing: genuine Frigidaire electronic oven controller; fitment not stated (2nd pass)</t>
         </is>
       </c>
     </row>
@@ -12396,15 +12416,19 @@
           <t>MGC64258906</t>
         </is>
       </c>
-      <c r="C495" s="2" t="inlineStr"/>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>LG Range Control Panel - MGC64258906</t>
+        </is>
+      </c>
       <c r="D495" s="2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E495" s="2" t="inlineStr">
         <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+          <t>lgparts.com listing: range control panel; no spec detail (2nd pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1: third pass adds 1 title
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -3765,25 +3765,29 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="inlineStr">
+      <c r="A136" s="3" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B136" s="3" t="inlineStr">
         <is>
           <t>DG94-01649A</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr"/>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Wall Oven Door Assembly - DG94-01649A</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing: wall oven door assembly (frame and glass); DG94-01649B is a separate listing (2nd pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1/Book2: more titles from extended search pass
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -671,25 +671,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>AGU75049015</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Upper Plate Assembly - AGU75049015</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>lgparts.com listing: upper plate assembly; fitment not stated (3rd pass); sheet brand "GE" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
@@ -829,48 +833,56 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>WB27X21183</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Panel Assembly - WB27X21183</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply exact-number listing: control panel assembly for range (3rd pass); sheet brand "Whirlpool" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>WB27X21183</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>GE Range Control Panel Assembly - WB27X21183</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>HD Supply exact-number listing: control panel assembly for range (3rd pass); sheet brand "Samsung" differs from part-number brand "GE"</t>
         </is>
       </c>
     </row>
@@ -1975,25 +1987,29 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>DE96-01027B</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Range Touch Control Panel - DE96-01027B</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>samsungparts.com listing: range touch control panel (sibling suffixes list other appliance types) (3rd pass)</t>
         </is>
       </c>
     </row>
@@ -2071,48 +2087,56 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>AGM30025504</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>LG Range Control Panel - AGM30025504</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>lgparts.com listing: range control panel (3rd pass); sheet brand "Samsung" differs from part-number brand "LG"</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>DG47-00048C</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr"/>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Microwave Oven Steam Heater - DG47-00048C</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>HnK Parts listing: steam heater for Samsung microwave oven (3rd pass)</t>
         </is>
       </c>
     </row>
@@ -4083,15 +4107,19 @@
           <t>DG90-01193A</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr"/>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Drawer Main Module Assembly - DG90-01193A</t>
+        </is>
+      </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+          <t>samsungparts.com listing: assembly drawer main module; appliance type not stated (3rd pass)</t>
         </is>
       </c>
     </row>
@@ -5923,25 +5951,29 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="inlineStr">
+      <c r="A222" s="3" t="inlineStr">
         <is>
           <t>Bertazzoni</t>
         </is>
       </c>
-      <c r="B222" s="2" t="inlineStr">
+      <c r="B222" s="3" t="inlineStr">
         <is>
           <t>DG94-01301G</t>
         </is>
       </c>
-      <c r="C222" s="2" t="inlineStr"/>
-      <c r="D222" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E222" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Range Main Top - DG94-01301G</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>samsungparts.com range and oven collection lists it as Range Main Top (3rd pass); sheet brand "Bertazzoni" differs from part-number brand "Samsung"</t>
         </is>
       </c>
     </row>
@@ -8165,15 +8197,19 @@
           <t>318185731</t>
         </is>
       </c>
-      <c r="C314" s="2" t="inlineStr"/>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Clock/Timer - 318185731</t>
+        </is>
+      </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+          <t>Third-party reseller listings only (two mirror sites); appliance type not stated (3rd pass)</t>
         </is>
       </c>
     </row>
@@ -8251,48 +8287,56 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="inlineStr">
+      <c r="A318" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B318" s="2" t="inlineStr">
+      <c r="B318" s="3" t="inlineStr">
         <is>
           <t>316630003</t>
         </is>
       </c>
-      <c r="C318" s="2" t="inlineStr"/>
-      <c r="D318" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E318" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Wall Oven Electronic Controller - 316630003</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing: genuine Frigidaire wall oven electronic controller (3rd pass); sheet brand "GE" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="inlineStr">
+      <c r="A319" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B319" s="2" t="inlineStr">
+      <c r="B319" s="3" t="inlineStr">
         <is>
           <t>316630005</t>
         </is>
       </c>
-      <c r="C319" s="2" t="inlineStr"/>
-      <c r="D319" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E319" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Wall Oven Gas Electronic Controller - 316630005</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing title: Frigidaire free-standing wall oven gas electronic controller (3rd pass); sheet brand "GE" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -8562,25 +8606,29 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="inlineStr">
+      <c r="A331" s="3" t="inlineStr">
         <is>
           <t>Frigidaire</t>
         </is>
       </c>
-      <c r="B331" s="2" t="inlineStr">
+      <c r="B331" s="3" t="inlineStr">
         <is>
           <t>316282991</t>
         </is>
       </c>
-      <c r="C331" s="2" t="inlineStr"/>
-      <c r="D331" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E331" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C331" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Maintop Assembly - 316282991</t>
+        </is>
+      </c>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E331" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts listing: maintop assembly for Kenmore/Frigidaire electric ranges (3rd pass)</t>
         </is>
       </c>
     </row>
@@ -8631,25 +8679,29 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" s="2" t="inlineStr">
+      <c r="A334" s="3" t="inlineStr">
         <is>
           <t>Blomberg</t>
         </is>
       </c>
-      <c r="B334" s="2" t="inlineStr">
+      <c r="B334" s="3" t="inlineStr">
         <is>
           <t>5304513155</t>
         </is>
       </c>
-      <c r="C334" s="2" t="inlineStr"/>
-      <c r="D334" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E334" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C334" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Smoothtop Assembly (Black) - 5304513155</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr">
+        <is>
+          <t>Walmart listing: SMOOTHTOP,ASSEMBLY,BLACK (3rd pass); sheet brand "Blomberg" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -11599,25 +11651,29 @@
       </c>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="inlineStr">
+      <c r="A458" s="3" t="inlineStr">
         <is>
           <t>Electrolux</t>
         </is>
       </c>
-      <c r="B458" s="2" t="inlineStr">
+      <c r="B458" s="3" t="inlineStr">
         <is>
           <t>316630005</t>
         </is>
       </c>
-      <c r="C458" s="2" t="inlineStr"/>
-      <c r="D458" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E458" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C458" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Wall Oven Gas Electronic Controller - 316630005</t>
+        </is>
+      </c>
+      <c r="D458" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E458" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing title: Frigidaire free-standing wall oven gas electronic controller (3rd pass); sheet brand "Electrolux" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -11695,25 +11751,29 @@
       </c>
     </row>
     <row r="462">
-      <c r="A462" s="2" t="inlineStr">
+      <c r="A462" s="3" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="B462" s="2" t="inlineStr">
+      <c r="B462" s="3" t="inlineStr">
         <is>
           <t>316630003</t>
         </is>
       </c>
-      <c r="C462" s="2" t="inlineStr"/>
-      <c r="D462" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E462" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C462" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Wall Oven Electronic Controller - 316630003</t>
+        </is>
+      </c>
+      <c r="D462" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E462" s="3" t="inlineStr">
+        <is>
+          <t>iFixit listing: genuine Frigidaire wall oven electronic controller (3rd pass); sheet brand "GE" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -11751,15 +11811,19 @@
           <t>318185731</t>
         </is>
       </c>
-      <c r="C464" s="2" t="inlineStr"/>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>Frigidaire Clock/Timer - 318185731</t>
+        </is>
+      </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E464" s="2" t="inlineStr">
         <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+          <t>Third-party reseller listings only (two mirror sites); appliance type not stated (3rd pass); sheet brand "GE" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -11979,25 +12043,29 @@
       </c>
     </row>
     <row r="474">
-      <c r="A474" s="2" t="inlineStr">
+      <c r="A474" s="3" t="inlineStr">
         <is>
           <t>LG</t>
         </is>
       </c>
-      <c r="B474" s="2" t="inlineStr">
+      <c r="B474" s="3" t="inlineStr">
         <is>
           <t>5304513155</t>
         </is>
       </c>
-      <c r="C474" s="2" t="inlineStr"/>
-      <c r="D474" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E474" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Smoothtop Assembly (Black) - 5304513155</t>
+        </is>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>Walmart listing: SMOOTHTOP,ASSEMBLY,BLACK (3rd pass); sheet brand "LG" differs from part-number brand "Frigidaire"</t>
         </is>
       </c>
     </row>
@@ -12166,21 +12234,25 @@
       </c>
     </row>
     <row r="483">
-      <c r="A483" s="2" t="n"/>
-      <c r="B483" s="2" t="inlineStr">
+      <c r="A483" s="3" t="n"/>
+      <c r="B483" s="3" t="inlineStr">
         <is>
           <t>316282991</t>
         </is>
       </c>
-      <c r="C483" s="2" t="inlineStr"/>
-      <c r="D483" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E483" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C483" s="3" t="inlineStr">
+        <is>
+          <t>Frigidaire Range Maintop Assembly - 316282991</t>
+        </is>
+      </c>
+      <c r="D483" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E483" s="3" t="inlineStr">
+        <is>
+          <t>ereplacementparts listing: maintop assembly for Kenmore/Frigidaire electric ranges (3rd pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1/Book2: add 11020735 title
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -7491,25 +7491,29 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="inlineStr">
+      <c r="A286" s="3" t="inlineStr">
         <is>
           <t>Bosch</t>
         </is>
       </c>
-      <c r="B286" s="2" t="inlineStr">
+      <c r="B286" s="3" t="inlineStr">
         <is>
           <t>11020735</t>
         </is>
       </c>
-      <c r="C286" s="2" t="inlineStr"/>
-      <c r="D286" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E286" s="2" t="inlineStr">
-        <is>
-          <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>Bosch Wall Oven Control Board - 11020735</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E286" s="3" t="inlineStr">
+        <is>
+          <t>Sears PartsDirect exact-number listing: wall oven control board (replaces 00758196, 12006840); brand taken from sheet (4th pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Book1/Book2: add generic fallback title column for unidentified rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book1_H1_tags.xlsx
+++ b/Book1_H1_tags.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,11 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E500"/>
+  <dimension ref="A1:F500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -437,6 +443,7 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,6 +472,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Generic fallback title (unverified part type)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -488,6 +500,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB27X20745</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -511,6 +528,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB27X20745</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -615,6 +637,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WP71001872</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -908,6 +935,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10780927</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -931,6 +963,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - 211840P</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -954,6 +991,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - 211840P</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1004,6 +1046,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10206087</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1027,6 +1074,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10877558</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1050,6 +1102,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03575A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1154,6 +1211,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11122533</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1204,6 +1266,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10734609</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1227,6 +1294,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10894095</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1250,6 +1322,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10177195</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1354,6 +1431,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11099813</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1377,6 +1459,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11088878</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1562,6 +1649,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - AGM75549801</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1612,6 +1704,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10904901</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -1662,6 +1759,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE92-03967A</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1685,6 +1787,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG96-00427A</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1708,6 +1815,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE96-01050B</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1758,6 +1870,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01281B</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1781,6 +1898,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10453983</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -1831,6 +1953,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10572538</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -1881,6 +2008,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10636386</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -1958,6 +2090,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - AGU74969001</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2062,6 +2199,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10196405BU</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2085,6 +2227,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - MEB63654001</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -2162,6 +2309,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG67-00166A</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2185,6 +2337,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01961A</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2208,6 +2365,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG67-00152A</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2231,6 +2393,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01994A</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2254,6 +2421,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG82-01521A</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2277,6 +2449,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG82-01523A</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2300,6 +2477,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG81-04117A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2323,6 +2505,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04247B</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2346,6 +2533,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03701A</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2396,6 +2588,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01141E</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -2446,6 +2643,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01727C</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2469,6 +2671,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG96-00728A</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -2519,6 +2726,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-02881D</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2569,6 +2781,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03551K</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2592,6 +2809,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG96-00773L</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2615,6 +2837,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01358D</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2692,6 +2919,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03552C</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -2742,6 +2974,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-02896A</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2765,6 +3002,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01193C</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2788,6 +3030,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01232B</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2811,6 +3058,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04664L</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2861,6 +3113,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01184C</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2911,6 +3168,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04664B</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -2961,6 +3223,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-05016A</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2984,6 +3251,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-02881C</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3007,6 +3279,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03551D</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3030,6 +3307,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE81-04440A</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3053,6 +3335,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04664H</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3076,6 +3363,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03952T</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3099,6 +3391,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01232A</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3122,6 +3419,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04148C</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3226,6 +3528,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE81-04441A</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3249,6 +3556,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE81-03806A</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3380,6 +3692,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - AHB73129211</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3403,6 +3720,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - AGU75049016</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3426,6 +3748,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG98-01358A</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3449,6 +3776,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE81-06920A</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3472,6 +3804,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11297273</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3495,6 +3832,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10908095</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3518,6 +3860,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11091927</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3541,6 +3888,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10804319</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -3618,6 +3970,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10877560</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3641,6 +3998,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10872562</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3664,6 +4026,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10336325</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3687,6 +4054,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04293A</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
@@ -3737,6 +4109,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03584A</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3760,6 +4137,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03580B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -3864,6 +4246,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-00513A</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -4022,6 +4409,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F144" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04108B</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -4072,6 +4464,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01301C</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -4095,6 +4492,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F147" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG96-00528A</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -4145,6 +4547,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03551C</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4168,6 +4575,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03551A</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -4218,6 +4630,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03552K</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -4268,6 +4685,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03598B</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -4291,6 +4713,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F155" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE94-05320A</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -4395,6 +4822,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-05016D</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -4418,6 +4850,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-02672A</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -4468,6 +4905,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03549N</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -4491,6 +4933,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F163" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03952W</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -4514,6 +4961,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F164" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03952P</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -4537,6 +4989,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F165" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03577D</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -4560,6 +5017,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE94-05062B</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -4583,6 +5045,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F167" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03580A</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -4633,6 +5100,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F169" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01727E</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -4656,6 +5128,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-03982A</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -4679,6 +5156,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F171" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE94-05062C</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -4702,6 +5184,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG90-01184A</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -4725,6 +5212,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F173" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04089A</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -4748,6 +5240,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10254671</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4771,6 +5268,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F175" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10472038</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -4794,6 +5296,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10340694</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -4844,6 +5351,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F178" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10550508</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -5029,6 +5541,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F185" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10314422</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -5052,6 +5569,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W10314419</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -5129,6 +5651,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F189" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WPW10271737</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
@@ -5233,6 +5760,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WP8507P226-60</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -5256,6 +5788,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F194" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE92-02439F</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -5333,6 +5870,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F197" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - MEE62306301</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -5545,6 +6087,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F205" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04148E</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -5595,6 +6142,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F207" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DE81-04526A</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
@@ -5672,6 +6224,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F210" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11295990</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -5695,6 +6252,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F211" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - EBR87050404</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -5718,6 +6280,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - EBR87050401</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -5741,6 +6308,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F213" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - EBR85707901</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -5791,6 +6363,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F215" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01301E</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
@@ -5922,6 +6499,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F220" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - W11122531</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -5999,6 +6581,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F223" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG92-01198F</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -6022,6 +6609,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F224" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01548B</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -6045,6 +6637,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F225" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-01545B</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -6095,6 +6692,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F227" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Replacement Part - DG94-04664P</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -6118,6 +6720,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F228" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - Z350251</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
@@ -6195,6 +6802,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F231" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 409047</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -6218,6 +6830,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F232" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125320</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
@@ -6268,6 +6885,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F234" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125190</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -6291,6 +6913,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F235" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125158</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -6314,6 +6941,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F236" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128006-DA</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -6337,6 +6969,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F237" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 1080923-DA</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -6360,6 +6997,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F238" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 1080921-DA</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -6383,6 +7025,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F239" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 128017-DA</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -6406,6 +7053,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F240" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 128023-DA</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -6429,6 +7081,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F241" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 128032-DA</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -6452,6 +7109,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F242" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 200560</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -6475,6 +7137,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F243" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 128019</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -6498,6 +7165,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F244" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 200558</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -6548,6 +7220,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F246" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - Z180301</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -6571,6 +7248,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F247" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 125194</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -6621,6 +7303,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F249" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 1081047</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -6644,6 +7331,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F250" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 1081068</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -6667,6 +7359,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F251" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 11036753</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -6690,6 +7387,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F252" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 11031383</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -6713,6 +7415,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F253" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 681176</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -6736,6 +7443,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F254" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 267600065</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -6759,6 +7471,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F255" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 210600165</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -6782,6 +7499,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F256" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 771361</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -6832,6 +7554,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F258" s="4" t="inlineStr">
+        <is>
+          <t>Fisher &amp; Paykel Replacement Part - 716392</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
@@ -6882,6 +7609,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F260" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 12026566</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
@@ -6932,6 +7664,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F262" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 626726</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -6955,6 +7692,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F263" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 683860</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -6978,6 +7720,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F264" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 449489</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -7001,6 +7748,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F265" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318261301</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -7024,6 +7776,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F266" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 808751511</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -7047,6 +7804,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F267" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304508977</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="3" t="inlineStr">
@@ -7097,6 +7859,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F269" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 676872</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -7120,6 +7887,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F270" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304495522</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -7143,6 +7915,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F271" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304495521</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="3" t="inlineStr">
@@ -7274,6 +8051,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F276" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304503761</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -7324,6 +8106,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F278" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 649265</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -7347,6 +8134,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F279" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 709785</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -7370,6 +8162,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F280" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 618624</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -7393,6 +8190,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F281" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 12012946</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -7416,6 +8218,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F282" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304511178</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -7439,6 +8246,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F283" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 12011384</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="3" t="inlineStr">
@@ -7489,6 +8301,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F285" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 709786</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="3" t="inlineStr">
@@ -7539,6 +8356,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F287" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 11020740</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -7562,6 +8384,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F288" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 11020743</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -7585,6 +8412,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F289" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 798846</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -7608,6 +8440,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F290" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316472803</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="3" t="inlineStr">
@@ -7739,6 +8576,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F295" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 12028039</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -7762,6 +8604,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F296" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - 12009513</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -7785,6 +8632,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F297" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304524907</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="3" t="inlineStr">
@@ -7835,6 +8687,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F299" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 12035575</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -7858,6 +8715,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F300" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 12035570</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="3" t="inlineStr">
@@ -7962,6 +8824,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F304" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316418501</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -7985,6 +8852,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F305" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318258201</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
@@ -8008,6 +8880,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F306" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316456238</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -8031,6 +8908,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F307" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318022001</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="3" t="inlineStr">
@@ -8162,6 +9044,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F312" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB57K10128</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="3" t="inlineStr">
@@ -8266,6 +9153,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F316" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316531960</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
@@ -8289,6 +9181,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F317" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316650003</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="3" t="inlineStr">
@@ -8366,6 +9263,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F320" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462865</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -8389,6 +9291,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F321" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462890</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -8412,6 +9319,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F322" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316453036</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -8435,6 +9347,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F323" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316531983</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="3" t="inlineStr">
@@ -8512,6 +9429,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F326" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462878</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="3" t="inlineStr">
@@ -8562,6 +9484,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F328" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316630001</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -8585,6 +9512,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F329" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316650001</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -8608,6 +9540,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F330" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316630004</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="3" t="inlineStr">
@@ -8658,6 +9595,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F332" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316442118</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -8681,6 +9623,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F333" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304514991</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="3" t="inlineStr">
@@ -8731,6 +9678,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F335" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513222</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -8754,6 +9706,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F336" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304514197</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -8777,6 +9734,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F337" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB48X23580</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="3" t="inlineStr">
@@ -8962,6 +9924,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F344" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513242</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -8985,6 +9952,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F345" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304515481</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -9008,6 +9980,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F346" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 4410600043</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="3" t="inlineStr">
@@ -9058,6 +10035,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F348" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304522786</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="3" t="inlineStr">
@@ -9108,6 +10090,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F350" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304519397</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -9131,6 +10118,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F351" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513844</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="3" t="inlineStr">
@@ -9181,6 +10173,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F353" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 210600164</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="3" t="inlineStr">
@@ -9231,6 +10228,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F355" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 669416</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
@@ -9254,6 +10256,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F356" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 20001930</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -9277,6 +10284,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F357" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 749003</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="3" t="inlineStr">
@@ -9327,6 +10339,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F359" s="4" t="inlineStr">
+        <is>
+          <t>Bosch Replacement Part - 4410600082</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="3" t="inlineStr">
@@ -9404,6 +10421,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F362" s="4" t="inlineStr">
+        <is>
+          <t>Whirlpool Replacement Part - WP6610457</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
@@ -9427,6 +10449,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F363" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 772646</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
@@ -9450,6 +10477,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F364" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 20004767</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
@@ -9473,6 +10505,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F365" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 10016262</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -9496,6 +10533,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F366" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 10016259</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
@@ -9519,6 +10561,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F367" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 11051367</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -9542,6 +10589,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F368" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 12046599</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
@@ -9565,6 +10617,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F369" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 23003198</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
@@ -9588,6 +10645,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F370" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 11019880</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
@@ -9611,6 +10673,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F371" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 681175</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
@@ -9634,6 +10701,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F372" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 703420</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
@@ -9657,6 +10729,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F373" s="4" t="inlineStr">
+        <is>
+          <t>Blomberg Replacement Part - 710664</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
@@ -9680,6 +10757,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F374" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 771592</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -9703,6 +10785,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F375" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 771648</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -9726,6 +10813,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F376" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 774642</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -9776,6 +10868,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F378" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 20000020</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="3" t="inlineStr">
@@ -9826,6 +10923,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F380" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 20000599</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
@@ -9849,6 +10951,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F381" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 673506</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
@@ -9872,6 +10979,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F382" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 659369</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
@@ -9895,6 +11007,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F383" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 210600498</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
@@ -9918,6 +11035,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F384" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 190264127</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
@@ -9941,6 +11063,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F385" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 210600551</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
@@ -9964,6 +11091,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F386" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 4410600086</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
@@ -9987,6 +11119,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F387" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 210600499</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
@@ -10010,6 +11147,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F388" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 260605048</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
@@ -10033,6 +11175,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F389" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 260605044</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
@@ -10056,6 +11203,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F390" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 210600217</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
@@ -10079,6 +11231,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F391" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 210600402</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
@@ -10102,6 +11259,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F392" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 267600066</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
@@ -10125,6 +11287,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F393" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 267600080</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
@@ -10148,6 +11315,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F394" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128006</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
@@ -10171,6 +11343,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F395" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128023</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
@@ -10194,6 +11371,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F396" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128036</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
@@ -10217,6 +11399,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F397" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128021</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
@@ -10240,6 +11427,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F398" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128026</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
@@ -10263,6 +11455,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F399" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128003</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="3" t="inlineStr">
@@ -10313,6 +11510,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F401" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128035</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
@@ -10336,6 +11538,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F402" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 1081013</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
@@ -10359,6 +11566,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F403" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 1081082</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
@@ -10382,6 +11594,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F404" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128010</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
@@ -10405,6 +11622,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F405" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128025</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="3" t="inlineStr">
@@ -10455,6 +11677,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F407" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128036-DA</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
@@ -10478,6 +11705,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F408" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128026-DA</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
@@ -10528,6 +11760,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F410" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 1081065</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
@@ -10551,6 +11788,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F411" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 1080943-DA</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
@@ -10574,6 +11816,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F412" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 128024-DA</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
@@ -10597,6 +11844,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F413" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 211258</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
@@ -10620,6 +11872,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F414" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - Z160143</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
@@ -10670,6 +11927,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F416" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125133</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
@@ -10693,6 +11955,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F417" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125153</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
@@ -10743,6 +12010,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F419" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125319</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
@@ -10766,6 +12038,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F420" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125335</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
@@ -10789,6 +12066,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F421" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125134</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
@@ -10812,6 +12094,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F422" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125345</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
@@ -10835,6 +12122,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F423" s="4" t="inlineStr">
+        <is>
+          <t>Bertazzoni Replacement Part - 125322</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
@@ -10885,6 +12177,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F425" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125170</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" s="3" t="inlineStr">
@@ -10935,6 +12232,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F427" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125309</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
@@ -10958,6 +12260,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F428" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125321</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
@@ -10981,6 +12288,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F429" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125341</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
@@ -11004,6 +12316,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F430" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125346</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
@@ -11027,6 +12344,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F431" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 200536</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
@@ -11050,6 +12372,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F432" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125162</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
@@ -11073,6 +12400,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F433" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125187</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
@@ -11123,6 +12455,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F435" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125317</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
@@ -11146,6 +12483,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F436" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125323</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
@@ -11169,6 +12511,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F437" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125307</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
@@ -11192,6 +12539,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F438" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125318</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
@@ -11215,6 +12567,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F439" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 410701</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
@@ -11265,6 +12622,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F441" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 125339</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
@@ -11315,6 +12677,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F443" s="4" t="inlineStr">
+        <is>
+          <t>Electrolux Replacement Part - 1080442</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="3" t="inlineStr">
@@ -11365,6 +12732,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F445" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316418501</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
@@ -11388,6 +12760,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F446" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316442118</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="3" t="inlineStr">
@@ -11438,6 +12815,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F448" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316456238</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="3" t="inlineStr">
@@ -11488,6 +12870,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F450" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462890</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
@@ -11511,6 +12898,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F451" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316472803</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
@@ -11534,6 +12926,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F452" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316453036</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
@@ -11557,6 +12954,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F453" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316531983</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
@@ -11580,6 +12982,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F454" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462865</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
@@ -11603,6 +13010,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F455" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316462878</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
@@ -11626,6 +13038,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F456" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316531960</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="3" t="inlineStr">
@@ -11730,6 +13147,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F460" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316650001</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
@@ -11753,6 +13175,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F461" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316630004</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="3" t="inlineStr">
@@ -11803,6 +13230,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F463" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316630001</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
@@ -11853,6 +13285,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F465" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318022001</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
@@ -11876,6 +13313,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F466" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318258201</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
@@ -11899,6 +13341,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F467" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 318261301</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
@@ -11949,6 +13396,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F469" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304495522</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
@@ -11972,6 +13424,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F470" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304503761</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
@@ -11995,6 +13452,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F471" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304508977</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
@@ -12018,6 +13480,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F472" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304511178</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="3" t="inlineStr">
@@ -12095,6 +13562,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F475" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513242</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
@@ -12116,6 +13588,11 @@
       <c r="E476" s="2" t="inlineStr">
         <is>
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+        </is>
+      </c>
+      <c r="F476" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513222</t>
         </is>
       </c>
     </row>
@@ -12137,6 +13614,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F477" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304514197</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n"/>
@@ -12156,6 +13638,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F478" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304514991</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n"/>
@@ -12175,6 +13662,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F479" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304519397</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n"/>
@@ -12194,6 +13686,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F480" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304524907</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n"/>
@@ -12236,6 +13733,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F482" s="4" t="inlineStr">
+        <is>
+          <t>None Replacement Part - 808751511</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" s="3" t="n"/>
@@ -12370,6 +13872,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F488" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB56X25765</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n"/>
@@ -12389,6 +13896,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F489" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 316650003</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n"/>
@@ -12408,6 +13920,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F490" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304513844</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n"/>
@@ -12427,6 +13944,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F491" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304515481</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n"/>
@@ -12446,6 +13968,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F492" s="4" t="inlineStr">
+        <is>
+          <t>Frigidaire Replacement Part - 5304522786</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n"/>
@@ -12465,6 +13992,11 @@
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
         </is>
       </c>
+      <c r="F493" s="4" t="inlineStr">
+        <is>
+          <t>GE Replacement Part - WB27X43578</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" s="3" t="n"/>
@@ -12528,6 +14060,11 @@
       <c r="E496" s="2" t="inlineStr">
         <is>
           <t>No page found for this exact part number by web search; not confident enough to name the appliance/part</t>
+        </is>
+      </c>
+      <c r="F496" s="4" t="inlineStr">
+        <is>
+          <t>LG Replacement Part - MEB63654003</t>
         </is>
       </c>
     </row>

</xml_diff>